<commit_message>
Add Team Valuations board, per-team value chips, and Sports hub restructure
New /sports/valuations lists 187 teams (Forbes US leagues + Sportico global football) on a sortable, filterable board, each linking to its team page and league/country hub; lib/valuations.ts resolves rows via the shared resolveTeamLink. NFL/NBA/MLB/NHL/football team headers gain a clickable valuation chip that deep-links to the board. The Sports hub now leads with a Deep-Dives section (Team Valuations, The Team That Wins the City) plus on-this-page nav, then the league directory, then the map. Data extracted from the new Team Valuations sheet of OtherLeagues.xlsx via scripts/build-valuations-data.py.
</commit_message>
<xml_diff>
--- a/OtherLeagues.xlsx
+++ b/OtherLeagues.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a9fb27646cb5ea21/Excel Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="189" documentId="8_{595D2767-5E65-418A-8CBF-B9F1CB0B6B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D89EC4B7-FF01-40EE-A4D0-D78B7B275C35}"/>
+  <xr:revisionPtr revIDLastSave="196" documentId="8_{595D2767-5E65-418A-8CBF-B9F1CB0B6B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8D8F587-F54B-43E2-B854-ABC6C253AD03}"/>
   <bookViews>
-    <workbookView xWindow="8715" yWindow="810" windowWidth="36705" windowHeight="16800" activeTab="4" xr2:uid="{0A162ED7-1454-46DB-B884-8A00FDA340E5}"/>
+    <workbookView xWindow="6990" yWindow="345" windowWidth="30510" windowHeight="16845" activeTab="5" xr2:uid="{0A162ED7-1454-46DB-B884-8A00FDA340E5}"/>
   </bookViews>
   <sheets>
     <sheet name="IPL Table" sheetId="1" r:id="rId1"/>
@@ -18,10 +18,12 @@
     <sheet name="Euroleague Table" sheetId="3" r:id="rId3"/>
     <sheet name="Women's Club Football" sheetId="5" r:id="rId4"/>
     <sheet name="WNBA" sheetId="6" r:id="rId5"/>
+    <sheet name="Team Valuations" sheetId="8" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Euroleague Table'!$A$1:$S$1048</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'IPL Table'!$A$1:$N$167</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Team Valuations'!$A$1:$E$188</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10645" uniqueCount="751">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11211" uniqueCount="943">
   <si>
     <t>Pos</t>
   </si>
@@ -2300,19 +2302,596 @@
   </si>
   <si>
     <t>Defunct Teams</t>
+  </si>
+  <si>
+    <t>San Diego FC</t>
+  </si>
+  <si>
+    <t>St. Louis City SC</t>
+  </si>
+  <si>
+    <t>Charlotte FC</t>
+  </si>
+  <si>
+    <t>Austin FC</t>
+  </si>
+  <si>
+    <t>Nashville SC</t>
+  </si>
+  <si>
+    <t>Inter Miami CF</t>
+  </si>
+  <si>
+    <t>FC Cincinnati</t>
+  </si>
+  <si>
+    <t>Los Angeles FC</t>
+  </si>
+  <si>
+    <t>Minnesota United</t>
+  </si>
+  <si>
+    <t>Atlanta United</t>
+  </si>
+  <si>
+    <t>New York City FC</t>
+  </si>
+  <si>
+    <t>Portland Timbers</t>
+  </si>
+  <si>
+    <t>Philadelphia Union</t>
+  </si>
+  <si>
+    <t>Seattle Sounders FC</t>
+  </si>
+  <si>
+    <t>Toronto FC</t>
+  </si>
+  <si>
+    <t>Houston Dynamo</t>
+  </si>
+  <si>
+    <t>Chicago Fire</t>
+  </si>
+  <si>
+    <t>San Jose Earthquakes</t>
+  </si>
+  <si>
+    <t>Columbus Crew</t>
+  </si>
+  <si>
+    <t>New York Red Bulls</t>
+  </si>
+  <si>
+    <t>Sporting Kansas City</t>
+  </si>
+  <si>
+    <t>DC United</t>
+  </si>
+  <si>
+    <t>Los Angeles Galaxy</t>
+  </si>
+  <si>
+    <t>Mexico</t>
+  </si>
+  <si>
+    <t>Monterrey</t>
+  </si>
+  <si>
+    <t>CF América</t>
+  </si>
+  <si>
+    <t>Chivas Guadalajara</t>
+  </si>
+  <si>
+    <t>Atlético de Madrid</t>
+  </si>
+  <si>
+    <t>Sevilla FC</t>
+  </si>
+  <si>
+    <t>FC Porto</t>
+  </si>
+  <si>
+    <t>Benfica</t>
+  </si>
+  <si>
+    <t>Juventus</t>
+  </si>
+  <si>
+    <t>Internazionale</t>
+  </si>
+  <si>
+    <t>Atalanta</t>
+  </si>
+  <si>
+    <t>Sportico, World's 50 Most Valuable Soccer Teams 2026 (Apr 22, 2026)</t>
+  </si>
+  <si>
+    <t>Lazio</t>
+  </si>
+  <si>
+    <t>AC Milan</t>
+  </si>
+  <si>
+    <t>AS Roma</t>
+  </si>
+  <si>
+    <t>RB Leipzig</t>
+  </si>
+  <si>
+    <t>Olympique Lyonnais</t>
+  </si>
+  <si>
+    <t>SSC Napoli</t>
+  </si>
+  <si>
+    <t>AFC Bournemouth</t>
+  </si>
+  <si>
+    <t>Sunderland</t>
+  </si>
+  <si>
+    <t>Leeds United</t>
+  </si>
+  <si>
+    <t>Brentford</t>
+  </si>
+  <si>
+    <t>Borussia Dortmund</t>
+  </si>
+  <si>
+    <t>Eintracht Frankfurt</t>
+  </si>
+  <si>
+    <t>Crystal Palace</t>
+  </si>
+  <si>
+    <t>Ajax</t>
+  </si>
+  <si>
+    <t>Bayern Munich</t>
+  </si>
+  <si>
+    <t>Paris Saint-Germain</t>
+  </si>
+  <si>
+    <t>Brighton &amp; Hove Albion</t>
+  </si>
+  <si>
+    <t>West Ham United</t>
+  </si>
+  <si>
+    <t>Everton</t>
+  </si>
+  <si>
+    <t>Newcastle United</t>
+  </si>
+  <si>
+    <t>Aston Villa</t>
+  </si>
+  <si>
+    <t>Forbes (1998-2025), via fanancialsports.com</t>
+  </si>
+  <si>
+    <t>MLB</t>
+  </si>
+  <si>
+    <t>Miami Marlins</t>
+  </si>
+  <si>
+    <t>Tampa Bay Rays</t>
+  </si>
+  <si>
+    <t>NHL</t>
+  </si>
+  <si>
+    <t>Columbus Blue Jackets</t>
+  </si>
+  <si>
+    <t>Tottenham Hotspur</t>
+  </si>
+  <si>
+    <t>Kansas City Royals</t>
+  </si>
+  <si>
+    <t>Buffalo Sabres</t>
+  </si>
+  <si>
+    <t>Chelsea</t>
+  </si>
+  <si>
+    <t>Cincinnati Reds</t>
+  </si>
+  <si>
+    <t>Winnipeg Jets</t>
+  </si>
+  <si>
+    <t>Pittsburgh Pirates</t>
+  </si>
+  <si>
+    <t>Ottawa Senators</t>
+  </si>
+  <si>
+    <t>Manchester United</t>
+  </si>
+  <si>
+    <t>Anaheim Ducks</t>
+  </si>
+  <si>
+    <t>Manchester City</t>
+  </si>
+  <si>
+    <t>Cleveland Guardians</t>
+  </si>
+  <si>
+    <t>Utah Mammoth</t>
+  </si>
+  <si>
+    <t>Colorado Rockies</t>
+  </si>
+  <si>
+    <t>San Jose Sharks</t>
+  </si>
+  <si>
+    <t>Minnesota Twins</t>
+  </si>
+  <si>
+    <t>Vegas Golden Knights</t>
+  </si>
+  <si>
+    <t>St. Louis Blues</t>
+  </si>
+  <si>
+    <t>Seattle Kraken</t>
+  </si>
+  <si>
+    <t>Detroit Tigers</t>
+  </si>
+  <si>
+    <t>Nashville Predators</t>
+  </si>
+  <si>
+    <t>Los Angeles Kings</t>
+  </si>
+  <si>
+    <t>Arizona Diamondbacks</t>
+  </si>
+  <si>
+    <t>Florida Panthers</t>
+  </si>
+  <si>
+    <t>Milwaukee Brewers</t>
+  </si>
+  <si>
+    <t>Minnesota Wild</t>
+  </si>
+  <si>
+    <t>Pittsburgh Penguins</t>
+  </si>
+  <si>
+    <t>Dallas Stars</t>
+  </si>
+  <si>
+    <t>Colorado Avalanche</t>
+  </si>
+  <si>
+    <t>Athletics</t>
+  </si>
+  <si>
+    <t>Chicago Blackhawks</t>
+  </si>
+  <si>
+    <t>Vancouver Canucks</t>
+  </si>
+  <si>
+    <t>Edmonton Oilers</t>
+  </si>
+  <si>
+    <t>Calgary Flames</t>
+  </si>
+  <si>
+    <t>Baltimore Orioles</t>
+  </si>
+  <si>
+    <t>Washington Capitals</t>
+  </si>
+  <si>
+    <t>San Diego Padres</t>
+  </si>
+  <si>
+    <t>Carolina Hurricanes</t>
+  </si>
+  <si>
+    <t>Philadelphia Flyers</t>
+  </si>
+  <si>
+    <t>Chicago White Sox</t>
+  </si>
+  <si>
+    <t>New York Rangers</t>
+  </si>
+  <si>
+    <t>Tampa Bay Lightning</t>
+  </si>
+  <si>
+    <t>New York Islanders</t>
+  </si>
+  <si>
+    <t>New Jersey Devils</t>
+  </si>
+  <si>
+    <t>Washington Nationals</t>
+  </si>
+  <si>
+    <t>Toronto Blue Jays</t>
+  </si>
+  <si>
+    <t>Detroit Red Wings</t>
+  </si>
+  <si>
+    <t>Seattle Mariners</t>
+  </si>
+  <si>
+    <t>Boston Bruins</t>
+  </si>
+  <si>
+    <t>Toronto Maple Leafs</t>
+  </si>
+  <si>
+    <t>Texas Rangers</t>
+  </si>
+  <si>
+    <t>Montreal Canadiens</t>
+  </si>
+  <si>
+    <t>NBA</t>
+  </si>
+  <si>
+    <t>San Antonio Spurs</t>
+  </si>
+  <si>
+    <t>New Orleans Pelicans</t>
+  </si>
+  <si>
+    <t>St. Louis Cardinals</t>
+  </si>
+  <si>
+    <t>Memphis Grizzlies</t>
+  </si>
+  <si>
+    <t>Houston Rockets</t>
+  </si>
+  <si>
+    <t>Los Angeles Angels</t>
+  </si>
+  <si>
+    <t>Dallas Mavericks</t>
+  </si>
+  <si>
+    <t>Sacramento Kings</t>
+  </si>
+  <si>
+    <t>Houston Astros</t>
+  </si>
+  <si>
+    <t>Phoenix Suns</t>
+  </si>
+  <si>
+    <t>Los Angeles Lakers</t>
+  </si>
+  <si>
+    <t>Atlanta Braves</t>
+  </si>
+  <si>
+    <t>Los Angeles Clippers</t>
+  </si>
+  <si>
+    <t>Golden State Warriors</t>
+  </si>
+  <si>
+    <t>Philadelphia Phillies</t>
+  </si>
+  <si>
+    <t>Utah Jazz</t>
+  </si>
+  <si>
+    <t>Portland Trail Blazers</t>
+  </si>
+  <si>
+    <t>New York Mets</t>
+  </si>
+  <si>
+    <t>Oklahoma City Thunder</t>
+  </si>
+  <si>
+    <t>Minnesota Timberwolves</t>
+  </si>
+  <si>
+    <t>Denver Nuggets</t>
+  </si>
+  <si>
+    <t>Washington Wizards</t>
+  </si>
+  <si>
+    <t>Orlando Magic</t>
+  </si>
+  <si>
+    <t>Miami Heat</t>
+  </si>
+  <si>
+    <t>Detroit Pistons</t>
+  </si>
+  <si>
+    <t>Charlotte Hornets</t>
+  </si>
+  <si>
+    <t>Atlanta Hawks</t>
+  </si>
+  <si>
+    <t>Milwaukee Bucks</t>
+  </si>
+  <si>
+    <t>Indiana Pacers</t>
+  </si>
+  <si>
+    <t>San Francisco Giants</t>
+  </si>
+  <si>
+    <t>Cleveland Cavaliers</t>
+  </si>
+  <si>
+    <t>Chicago Bulls</t>
+  </si>
+  <si>
+    <t>Philadelphia 76ers</t>
+  </si>
+  <si>
+    <t>New York Knicks</t>
+  </si>
+  <si>
+    <t>Brooklyn Nets</t>
+  </si>
+  <si>
+    <t>Boston Celtics</t>
+  </si>
+  <si>
+    <t>Toronto Raptors</t>
+  </si>
+  <si>
+    <t>Los Angeles Dodgers</t>
+  </si>
+  <si>
+    <t>Chicago Cubs</t>
+  </si>
+  <si>
+    <t>Boston Red Sox</t>
+  </si>
+  <si>
+    <t>NFL</t>
+  </si>
+  <si>
+    <t>Cincinnati Bengals</t>
+  </si>
+  <si>
+    <t>New Orleans Saints</t>
+  </si>
+  <si>
+    <t>Detroit Lions</t>
+  </si>
+  <si>
+    <t>Arizona Cardinals</t>
+  </si>
+  <si>
+    <t>Jacksonville Jaguars</t>
+  </si>
+  <si>
+    <t>Carolina Panthers</t>
+  </si>
+  <si>
+    <t>New York Yankees</t>
+  </si>
+  <si>
+    <t>Indianapolis Colts</t>
+  </si>
+  <si>
+    <t>Buffalo Bills</t>
+  </si>
+  <si>
+    <t>Los Angeles Chargers</t>
+  </si>
+  <si>
+    <t>Baltimore Ravens</t>
+  </si>
+  <si>
+    <t>Seattle Seahawks</t>
+  </si>
+  <si>
+    <t>Kansas City Chiefs</t>
+  </si>
+  <si>
+    <t>San Francisco 49ers</t>
+  </si>
+  <si>
+    <t>Minnesota Vikings</t>
+  </si>
+  <si>
+    <t>Los Angeles Rams</t>
+  </si>
+  <si>
+    <t>Tennessee Titans</t>
+  </si>
+  <si>
+    <t>Atlanta Falcons</t>
+  </si>
+  <si>
+    <t>Tampa Bay Buccaneers</t>
+  </si>
+  <si>
+    <t>Cleveland Browns</t>
+  </si>
+  <si>
+    <t>Pittsburgh Steelers</t>
+  </si>
+  <si>
+    <t>Green Bay Packers</t>
+  </si>
+  <si>
+    <t>Chicago Bears</t>
+  </si>
+  <si>
+    <t>Washington Commanders</t>
+  </si>
+  <si>
+    <t>Denver Broncos</t>
+  </si>
+  <si>
+    <t>Philadelphia Eagles</t>
+  </si>
+  <si>
+    <t>New York Giants</t>
+  </si>
+  <si>
+    <t>Houston Texans</t>
+  </si>
+  <si>
+    <t>Dallas Cowboys</t>
+  </si>
+  <si>
+    <t>Miami Dolphins</t>
+  </si>
+  <si>
+    <t>Las Vegas Raiders</t>
+  </si>
+  <si>
+    <t>New York Jets</t>
+  </si>
+  <si>
+    <t>New England Patriots</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>Value ($M)</t>
+  </si>
+  <si>
+    <t>Year</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0;\-0.0;&quot;-&quot;"/>
     <numFmt numFmtId="167" formatCode="0;\-0;&quot;&quot;"/>
+    <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2395,8 +2974,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2421,6 +3007,11 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F3864"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -2439,7 +3030,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2491,6 +3082,16 @@
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="12" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -2610,10 +3211,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -70269,4 +70866,3217 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89D9355A-DA33-493A-90CE-7FBEA6A424DB}">
+  <dimension ref="A1:E188"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" customWidth="1"/>
+    <col min="4" max="4" width="13" style="34" customWidth="1"/>
+    <col min="5" max="5" width="61.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="38" t="s">
+        <v>942</v>
+      </c>
+      <c r="B1" s="38" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="38" t="s">
+        <v>135</v>
+      </c>
+      <c r="D1" s="39" t="s">
+        <v>941</v>
+      </c>
+      <c r="E1" s="38" t="s">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B2" s="35" t="s">
+        <v>935</v>
+      </c>
+      <c r="C2" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D2" s="36">
+        <v>13000</v>
+      </c>
+      <c r="E2" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B3" s="35" t="s">
+        <v>879</v>
+      </c>
+      <c r="C3" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D3" s="36">
+        <v>11000</v>
+      </c>
+      <c r="E3" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B4" s="35" t="s">
+        <v>922</v>
+      </c>
+      <c r="C4" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D4" s="36">
+        <v>10500</v>
+      </c>
+      <c r="E4" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B5" s="35" t="s">
+        <v>933</v>
+      </c>
+      <c r="C5" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D5" s="36">
+        <v>10100</v>
+      </c>
+      <c r="E5" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B6" s="35" t="s">
+        <v>876</v>
+      </c>
+      <c r="C6" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D6" s="36">
+        <v>10000</v>
+      </c>
+      <c r="E6" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B7" s="35" t="s">
+        <v>899</v>
+      </c>
+      <c r="C7" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D7" s="36">
+        <v>9750</v>
+      </c>
+      <c r="E7" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B8" s="35" t="s">
+        <v>939</v>
+      </c>
+      <c r="C8" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D8" s="36">
+        <v>9000</v>
+      </c>
+      <c r="E8" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B9" s="35" t="s">
+        <v>920</v>
+      </c>
+      <c r="C9" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D9" s="36">
+        <v>8600</v>
+      </c>
+      <c r="E9" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B10" s="35" t="s">
+        <v>932</v>
+      </c>
+      <c r="C10" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D10" s="36">
+        <v>8300</v>
+      </c>
+      <c r="E10" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B11" s="35" t="s">
+        <v>913</v>
+      </c>
+      <c r="C11" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D11" s="36">
+        <v>8200</v>
+      </c>
+      <c r="E11" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B12" s="35" t="s">
+        <v>929</v>
+      </c>
+      <c r="C12" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D12" s="36">
+        <v>8200</v>
+      </c>
+      <c r="E12" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B13" s="35" t="s">
+        <v>938</v>
+      </c>
+      <c r="C13" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D13" s="36">
+        <v>8100</v>
+      </c>
+      <c r="E13" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B14" s="35" t="s">
+        <v>937</v>
+      </c>
+      <c r="C14" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D14" s="36">
+        <v>7700</v>
+      </c>
+      <c r="E14" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B15" s="35" t="s">
+        <v>534</v>
+      </c>
+      <c r="C15" s="35" t="s">
+        <v>154</v>
+      </c>
+      <c r="D15" s="36">
+        <v>7700</v>
+      </c>
+      <c r="E15" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B16" s="35" t="s">
+        <v>930</v>
+      </c>
+      <c r="C16" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D16" s="36">
+        <v>7600</v>
+      </c>
+      <c r="E16" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B17" s="35" t="s">
+        <v>878</v>
+      </c>
+      <c r="C17" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D17" s="36">
+        <v>7500</v>
+      </c>
+      <c r="E17" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B18" s="35" t="s">
+        <v>936</v>
+      </c>
+      <c r="C18" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D18" s="36">
+        <v>7500</v>
+      </c>
+      <c r="E18" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B19" s="35" t="s">
+        <v>934</v>
+      </c>
+      <c r="C19" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D19" s="36">
+        <v>7400</v>
+      </c>
+      <c r="E19" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B20" s="35" t="s">
+        <v>903</v>
+      </c>
+      <c r="C20" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D20" s="36">
+        <v>6800</v>
+      </c>
+      <c r="E20" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B21" s="35" t="s">
+        <v>931</v>
+      </c>
+      <c r="C21" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D21" s="36">
+        <v>6800</v>
+      </c>
+      <c r="E21" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B22" s="35" t="s">
+        <v>901</v>
+      </c>
+      <c r="C22" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D22" s="36">
+        <v>6700</v>
+      </c>
+      <c r="E22" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B23" s="35" t="s">
+        <v>918</v>
+      </c>
+      <c r="C23" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D23" s="36">
+        <v>6700</v>
+      </c>
+      <c r="E23" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B24" s="35" t="s">
+        <v>928</v>
+      </c>
+      <c r="C24" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D24" s="36">
+        <v>6650</v>
+      </c>
+      <c r="E24" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B25" s="35" t="s">
+        <v>537</v>
+      </c>
+      <c r="C25" s="35" t="s">
+        <v>154</v>
+      </c>
+      <c r="D25" s="36">
+        <v>6650</v>
+      </c>
+      <c r="E25" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B26" s="35" t="s">
+        <v>925</v>
+      </c>
+      <c r="C26" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D26" s="36">
+        <v>6600</v>
+      </c>
+      <c r="E26" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B27" s="35" t="s">
+        <v>927</v>
+      </c>
+      <c r="C27" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D27" s="36">
+        <v>6500</v>
+      </c>
+      <c r="E27" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B28" s="35" t="s">
+        <v>821</v>
+      </c>
+      <c r="C28" s="35" t="s">
+        <v>376</v>
+      </c>
+      <c r="D28" s="36">
+        <v>6470</v>
+      </c>
+      <c r="E28" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B29" s="35" t="s">
+        <v>926</v>
+      </c>
+      <c r="C29" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D29" s="36">
+        <v>6400</v>
+      </c>
+      <c r="E29" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B30" s="35" t="s">
+        <v>924</v>
+      </c>
+      <c r="C30" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D30" s="36">
+        <v>6350</v>
+      </c>
+      <c r="E30" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B31" s="35" t="s">
+        <v>923</v>
+      </c>
+      <c r="C31" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D31" s="36">
+        <v>6300</v>
+      </c>
+      <c r="E31" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B32" s="35" t="s">
+        <v>921</v>
+      </c>
+      <c r="C32" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D32" s="36">
+        <v>6250</v>
+      </c>
+      <c r="E32" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B33" s="35" t="s">
+        <v>919</v>
+      </c>
+      <c r="C33" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D33" s="36">
+        <v>6200</v>
+      </c>
+      <c r="E33" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B34" s="35" t="s">
+        <v>917</v>
+      </c>
+      <c r="C34" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D34" s="36">
+        <v>6100</v>
+      </c>
+      <c r="E34" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B35" s="35" t="s">
+        <v>897</v>
+      </c>
+      <c r="C35" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D35" s="36">
+        <v>6000</v>
+      </c>
+      <c r="E35" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B36" s="35" t="s">
+        <v>916</v>
+      </c>
+      <c r="C36" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D36" s="36">
+        <v>6000</v>
+      </c>
+      <c r="E36" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B37" s="35" t="s">
+        <v>915</v>
+      </c>
+      <c r="C37" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D37" s="36">
+        <v>5950</v>
+      </c>
+      <c r="E37" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B38" s="35" t="s">
+        <v>870</v>
+      </c>
+      <c r="C38" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D38" s="36">
+        <v>5900</v>
+      </c>
+      <c r="E38" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B39" s="35" t="s">
+        <v>914</v>
+      </c>
+      <c r="C39" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D39" s="36">
+        <v>5900</v>
+      </c>
+      <c r="E39" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B40" s="35" t="s">
+        <v>800</v>
+      </c>
+      <c r="C40" s="35" t="s">
+        <v>173</v>
+      </c>
+      <c r="D40" s="36">
+        <v>5780</v>
+      </c>
+      <c r="E40" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B41" s="35" t="s">
+        <v>588</v>
+      </c>
+      <c r="C41" s="35" t="s">
+        <v>376</v>
+      </c>
+      <c r="D41" s="36">
+        <v>5740</v>
+      </c>
+      <c r="E41" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B42" s="35" t="s">
+        <v>889</v>
+      </c>
+      <c r="C42" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D42" s="36">
+        <v>5700</v>
+      </c>
+      <c r="E42" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B43" s="35" t="s">
+        <v>912</v>
+      </c>
+      <c r="C43" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D43" s="36">
+        <v>5700</v>
+      </c>
+      <c r="E43" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B44" s="35" t="s">
+        <v>823</v>
+      </c>
+      <c r="C44" s="35" t="s">
+        <v>376</v>
+      </c>
+      <c r="D44" s="36">
+        <v>5700</v>
+      </c>
+      <c r="E44" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B45" s="35" t="s">
+        <v>900</v>
+      </c>
+      <c r="C45" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D45" s="36">
+        <v>5600</v>
+      </c>
+      <c r="E45" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B46" s="35" t="s">
+        <v>911</v>
+      </c>
+      <c r="C46" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D46" s="36">
+        <v>5600</v>
+      </c>
+      <c r="E46" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B47" s="35" t="s">
+        <v>910</v>
+      </c>
+      <c r="C47" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D47" s="36">
+        <v>5500</v>
+      </c>
+      <c r="E47" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B48" s="35" t="s">
+        <v>898</v>
+      </c>
+      <c r="C48" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D48" s="36">
+        <v>5450</v>
+      </c>
+      <c r="E48" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B49" s="35" t="s">
+        <v>587</v>
+      </c>
+      <c r="C49" s="35" t="s">
+        <v>376</v>
+      </c>
+      <c r="D49" s="36">
+        <v>5430</v>
+      </c>
+      <c r="E49" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B50" s="35" t="s">
+        <v>875</v>
+      </c>
+      <c r="C50" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D50" s="36">
+        <v>5425</v>
+      </c>
+      <c r="E50" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B51" s="35" t="s">
+        <v>902</v>
+      </c>
+      <c r="C51" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D51" s="36">
+        <v>5400</v>
+      </c>
+      <c r="E51" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B52" s="35" t="s">
+        <v>909</v>
+      </c>
+      <c r="C52" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D52" s="36">
+        <v>5400</v>
+      </c>
+      <c r="E52" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B53" s="35" t="s">
+        <v>908</v>
+      </c>
+      <c r="C53" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D53" s="36">
+        <v>5300</v>
+      </c>
+      <c r="E53" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B54" s="35" t="s">
+        <v>907</v>
+      </c>
+      <c r="C54" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="D54" s="36">
+        <v>5250</v>
+      </c>
+      <c r="E54" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B55" s="35" t="s">
+        <v>872</v>
+      </c>
+      <c r="C55" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D55" s="36">
+        <v>5100</v>
+      </c>
+      <c r="E55" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B56" s="35" t="s">
+        <v>892</v>
+      </c>
+      <c r="C56" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D56" s="36">
+        <v>5000</v>
+      </c>
+      <c r="E56" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B57" s="35" t="s">
+        <v>801</v>
+      </c>
+      <c r="C57" s="35" t="s">
+        <v>164</v>
+      </c>
+      <c r="D57" s="36">
+        <v>5000</v>
+      </c>
+      <c r="E57" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B58" s="35" t="s">
+        <v>905</v>
+      </c>
+      <c r="C58" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D58" s="36">
+        <v>4800</v>
+      </c>
+      <c r="E58" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B59" s="35" t="s">
+        <v>896</v>
+      </c>
+      <c r="C59" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D59" s="36">
+        <v>4800</v>
+      </c>
+      <c r="E59" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B60" s="35" t="s">
+        <v>887</v>
+      </c>
+      <c r="C60" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D60" s="36">
+        <v>4700</v>
+      </c>
+      <c r="E60" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B61" s="35" t="s">
+        <v>904</v>
+      </c>
+      <c r="C61" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D61" s="36">
+        <v>4600</v>
+      </c>
+      <c r="E61" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B62" s="35" t="s">
+        <v>886</v>
+      </c>
+      <c r="C62" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D62" s="36">
+        <v>4600</v>
+      </c>
+      <c r="E62" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B63" s="35" t="s">
+        <v>873</v>
+      </c>
+      <c r="C63" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D63" s="36">
+        <v>4450</v>
+      </c>
+      <c r="E63" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B64" s="35" t="s">
+        <v>866</v>
+      </c>
+      <c r="C64" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D64" s="36">
+        <v>4400</v>
+      </c>
+      <c r="E64" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B65" s="35" t="s">
+        <v>862</v>
+      </c>
+      <c r="C65" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D65" s="36">
+        <v>4400</v>
+      </c>
+      <c r="E65" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B66" s="35" t="s">
+        <v>884</v>
+      </c>
+      <c r="C66" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D66" s="36">
+        <v>4350</v>
+      </c>
+      <c r="E66" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B67" s="35" t="s">
+        <v>893</v>
+      </c>
+      <c r="C67" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D67" s="36">
+        <v>4300</v>
+      </c>
+      <c r="E67" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B68" s="35" t="s">
+        <v>882</v>
+      </c>
+      <c r="C68" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D68" s="36">
+        <v>4250</v>
+      </c>
+      <c r="E68" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B69" s="35" t="s">
+        <v>894</v>
+      </c>
+      <c r="C69" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D69" s="36">
+        <v>4200</v>
+      </c>
+      <c r="E69" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B70" s="35" t="s">
+        <v>881</v>
+      </c>
+      <c r="C70" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D70" s="36">
+        <v>4100</v>
+      </c>
+      <c r="E70" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B71" s="35" t="s">
+        <v>895</v>
+      </c>
+      <c r="C71" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D71" s="36">
+        <v>4000</v>
+      </c>
+      <c r="E71" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A72" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B72" s="35" t="s">
+        <v>853</v>
+      </c>
+      <c r="C72" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D72" s="36">
+        <v>4000</v>
+      </c>
+      <c r="E72" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B73" s="35" t="s">
+        <v>816</v>
+      </c>
+      <c r="C73" s="35" t="s">
+        <v>376</v>
+      </c>
+      <c r="D73" s="36">
+        <v>4000</v>
+      </c>
+      <c r="E73" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B74" s="35" t="s">
+        <v>888</v>
+      </c>
+      <c r="C74" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D74" s="36">
+        <v>3900</v>
+      </c>
+      <c r="E74" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B75" s="35" t="s">
+        <v>891</v>
+      </c>
+      <c r="C75" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D75" s="36">
+        <v>3800</v>
+      </c>
+      <c r="E75" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B76" s="35" t="s">
+        <v>890</v>
+      </c>
+      <c r="C76" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D76" s="36">
+        <v>3650</v>
+      </c>
+      <c r="E76" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B77" s="35" t="s">
+        <v>885</v>
+      </c>
+      <c r="C77" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D77" s="36">
+        <v>3600</v>
+      </c>
+      <c r="E77" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A78" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B78" s="35" t="s">
+        <v>867</v>
+      </c>
+      <c r="C78" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D78" s="36">
+        <v>3550</v>
+      </c>
+      <c r="E78" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A79" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B79" s="35" t="s">
+        <v>869</v>
+      </c>
+      <c r="C79" s="35" t="s">
+        <v>865</v>
+      </c>
+      <c r="D79" s="36">
+        <v>3500</v>
+      </c>
+      <c r="E79" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A80" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B80" s="35" t="s">
+        <v>813</v>
+      </c>
+      <c r="C80" s="35" t="s">
+        <v>376</v>
+      </c>
+      <c r="D80" s="36">
+        <v>3500</v>
+      </c>
+      <c r="E80" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B81" s="35" t="s">
+        <v>864</v>
+      </c>
+      <c r="C81" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D81" s="36">
+        <v>3400</v>
+      </c>
+      <c r="E81" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B82" s="35" t="s">
+        <v>883</v>
+      </c>
+      <c r="C82" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D82" s="36">
+        <v>3200</v>
+      </c>
+      <c r="E82" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B83" s="35" t="s">
+        <v>845</v>
+      </c>
+      <c r="C83" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D83" s="36">
+        <v>3200</v>
+      </c>
+      <c r="E83" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A84" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B84" s="35" t="s">
+        <v>880</v>
+      </c>
+      <c r="C84" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D84" s="36">
+        <v>3100</v>
+      </c>
+      <c r="E84" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A85" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B85" s="35" t="s">
+        <v>834</v>
+      </c>
+      <c r="C85" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D85" s="36">
+        <v>3100</v>
+      </c>
+      <c r="E85" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A86" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B86" s="35" t="s">
+        <v>877</v>
+      </c>
+      <c r="C86" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D86" s="36">
+        <v>3000</v>
+      </c>
+      <c r="E86" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A87" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B87" s="35" t="s">
+        <v>861</v>
+      </c>
+      <c r="C87" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D87" s="36">
+        <v>2900</v>
+      </c>
+      <c r="E87" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A88" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B88" s="35" t="s">
+        <v>874</v>
+      </c>
+      <c r="C88" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D88" s="36">
+        <v>2800</v>
+      </c>
+      <c r="E88" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A89" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B89" s="35" t="s">
+        <v>843</v>
+      </c>
+      <c r="C89" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D89" s="36">
+        <v>2800</v>
+      </c>
+      <c r="E89" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A90" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B90" s="35" t="s">
+        <v>871</v>
+      </c>
+      <c r="C90" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D90" s="36">
+        <v>2750</v>
+      </c>
+      <c r="E90" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A91" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B91" s="35" t="s">
+        <v>851</v>
+      </c>
+      <c r="C91" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D91" s="36">
+        <v>2700</v>
+      </c>
+      <c r="E91" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A92" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B92" s="35" t="s">
+        <v>868</v>
+      </c>
+      <c r="C92" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D92" s="36">
+        <v>2550</v>
+      </c>
+      <c r="E92" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A93" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B93" s="35" t="s">
+        <v>848</v>
+      </c>
+      <c r="C93" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D93" s="36">
+        <v>2550</v>
+      </c>
+      <c r="E93" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A94" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B94" s="35" t="s">
+        <v>859</v>
+      </c>
+      <c r="C94" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D94" s="36">
+        <v>2500</v>
+      </c>
+      <c r="E94" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A95" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B95" s="35" t="s">
+        <v>778</v>
+      </c>
+      <c r="C95" s="35" t="s">
+        <v>154</v>
+      </c>
+      <c r="D95" s="36">
+        <v>2500</v>
+      </c>
+      <c r="E95" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A96" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B96" s="35" t="s">
+        <v>863</v>
+      </c>
+      <c r="C96" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D96" s="36">
+        <v>2450</v>
+      </c>
+      <c r="E96" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A97" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B97" s="35" t="s">
+        <v>856</v>
+      </c>
+      <c r="C97" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D97" s="36">
+        <v>2400</v>
+      </c>
+      <c r="E97" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A98" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B98" s="35" t="s">
+        <v>840</v>
+      </c>
+      <c r="C98" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D98" s="36">
+        <v>2300</v>
+      </c>
+      <c r="E98" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A99" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B99" s="35" t="s">
+        <v>860</v>
+      </c>
+      <c r="C99" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D99" s="36">
+        <v>2200</v>
+      </c>
+      <c r="E99" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A100" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B100" s="35" t="s">
+        <v>829</v>
+      </c>
+      <c r="C100" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D100" s="36">
+        <v>2200</v>
+      </c>
+      <c r="E100" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A101" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B101" s="35" t="s">
+        <v>796</v>
+      </c>
+      <c r="C101" s="35" t="s">
+        <v>173</v>
+      </c>
+      <c r="D101" s="36">
+        <v>2170</v>
+      </c>
+      <c r="E101" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A102" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B102" s="35" t="s">
+        <v>858</v>
+      </c>
+      <c r="C102" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D102" s="36">
+        <v>2150</v>
+      </c>
+      <c r="E102" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A103" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B103" s="35" t="s">
+        <v>844</v>
+      </c>
+      <c r="C103" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D103" s="36">
+        <v>2150</v>
+      </c>
+      <c r="E103" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A104" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B104" s="35" t="s">
+        <v>857</v>
+      </c>
+      <c r="C104" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D104" s="36">
+        <v>2100</v>
+      </c>
+      <c r="E104" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A105" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B105" s="35" t="s">
+        <v>855</v>
+      </c>
+      <c r="C105" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D105" s="36">
+        <v>2100</v>
+      </c>
+      <c r="E105" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A106" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B106" s="35" t="s">
+        <v>854</v>
+      </c>
+      <c r="C106" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D106" s="36">
+        <v>2050</v>
+      </c>
+      <c r="E106" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A107" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B107" s="35" t="s">
+        <v>852</v>
+      </c>
+      <c r="C107" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D107" s="36">
+        <v>2000</v>
+      </c>
+      <c r="E107" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A108" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B108" s="35" t="s">
+        <v>850</v>
+      </c>
+      <c r="C108" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D108" s="36">
+        <v>2000</v>
+      </c>
+      <c r="E108" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A109" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B109" s="35" t="s">
+        <v>849</v>
+      </c>
+      <c r="C109" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D109" s="36">
+        <v>1950</v>
+      </c>
+      <c r="E109" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A110" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B110" s="35" t="s">
+        <v>841</v>
+      </c>
+      <c r="C110" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D110" s="36">
+        <v>1950</v>
+      </c>
+      <c r="E110" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A111" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B111" s="35" t="s">
+        <v>847</v>
+      </c>
+      <c r="C111" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D111" s="36">
+        <v>1900</v>
+      </c>
+      <c r="E111" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A112" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B112" s="35" t="s">
+        <v>846</v>
+      </c>
+      <c r="C112" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D112" s="36">
+        <v>1900</v>
+      </c>
+      <c r="E112" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A113" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B113" s="35" t="s">
+        <v>831</v>
+      </c>
+      <c r="C113" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D113" s="36">
+        <v>1850</v>
+      </c>
+      <c r="E113" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A114" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B114" s="35" t="s">
+        <v>782</v>
+      </c>
+      <c r="C114" s="35" t="s">
+        <v>171</v>
+      </c>
+      <c r="D114" s="36">
+        <v>1840</v>
+      </c>
+      <c r="E114" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A115" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B115" s="35" t="s">
+        <v>842</v>
+      </c>
+      <c r="C115" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D115" s="36">
+        <v>1800</v>
+      </c>
+      <c r="E115" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A116" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B116" s="35" t="s">
+        <v>838</v>
+      </c>
+      <c r="C116" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D116" s="36">
+        <v>1800</v>
+      </c>
+      <c r="E116" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A117" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B117" s="35" t="s">
+        <v>839</v>
+      </c>
+      <c r="C117" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D117" s="36">
+        <v>1750</v>
+      </c>
+      <c r="E117" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A118" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B118" s="35" t="s">
+        <v>837</v>
+      </c>
+      <c r="C118" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D118" s="36">
+        <v>1700</v>
+      </c>
+      <c r="E118" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A119" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B119" s="35" t="s">
+        <v>836</v>
+      </c>
+      <c r="C119" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D119" s="36">
+        <v>1700</v>
+      </c>
+      <c r="E119" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A120" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B120" s="35" t="s">
+        <v>787</v>
+      </c>
+      <c r="C120" s="35" t="s">
+        <v>171</v>
+      </c>
+      <c r="D120" s="36">
+        <v>1660</v>
+      </c>
+      <c r="E120" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A121" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B121" s="35" t="s">
+        <v>783</v>
+      </c>
+      <c r="C121" s="35" t="s">
+        <v>171</v>
+      </c>
+      <c r="D121" s="36">
+        <v>1620</v>
+      </c>
+      <c r="E121" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A122" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B122" s="35" t="s">
+        <v>835</v>
+      </c>
+      <c r="C122" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D122" s="36">
+        <v>1600</v>
+      </c>
+      <c r="E122" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A123" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B123" s="35" t="s">
+        <v>833</v>
+      </c>
+      <c r="C123" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D123" s="36">
+        <v>1600</v>
+      </c>
+      <c r="E123" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A124" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B124" s="35" t="s">
+        <v>832</v>
+      </c>
+      <c r="C124" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D124" s="36">
+        <v>1550</v>
+      </c>
+      <c r="E124" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A125" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B125" s="35" t="s">
+        <v>830</v>
+      </c>
+      <c r="C125" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D125" s="36">
+        <v>1550</v>
+      </c>
+      <c r="E125" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A126" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B126" s="35" t="s">
+        <v>828</v>
+      </c>
+      <c r="C126" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D126" s="36">
+        <v>1500</v>
+      </c>
+      <c r="E126" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A127" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B127" s="35" t="s">
+        <v>827</v>
+      </c>
+      <c r="C127" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D127" s="36">
+        <v>1500</v>
+      </c>
+      <c r="E127" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A128" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B128" s="35" t="s">
+        <v>826</v>
+      </c>
+      <c r="C128" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D128" s="36">
+        <v>1475</v>
+      </c>
+      <c r="E128" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A129" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B129" s="35" t="s">
+        <v>825</v>
+      </c>
+      <c r="C129" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D129" s="36">
+        <v>1450</v>
+      </c>
+      <c r="E129" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A130" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B130" s="35" t="s">
+        <v>756</v>
+      </c>
+      <c r="C130" s="35" t="s">
+        <v>660</v>
+      </c>
+      <c r="D130" s="36">
+        <v>1450</v>
+      </c>
+      <c r="E130" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A131" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B131" s="35" t="s">
+        <v>824</v>
+      </c>
+      <c r="C131" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D131" s="36">
+        <v>1400</v>
+      </c>
+      <c r="E131" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A132" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B132" s="35" t="s">
+        <v>822</v>
+      </c>
+      <c r="C132" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D132" s="36">
+        <v>1400</v>
+      </c>
+      <c r="E132" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A133" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B133" s="35" t="s">
+        <v>758</v>
+      </c>
+      <c r="C133" s="35" t="s">
+        <v>660</v>
+      </c>
+      <c r="D133" s="36">
+        <v>1400</v>
+      </c>
+      <c r="E133" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A134" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B134" s="35" t="s">
+        <v>820</v>
+      </c>
+      <c r="C134" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D134" s="36">
+        <v>1375</v>
+      </c>
+      <c r="E134" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A135" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B135" s="35" t="s">
+        <v>819</v>
+      </c>
+      <c r="C135" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D135" s="36">
+        <v>1350</v>
+      </c>
+      <c r="E135" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A136" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B136" s="35" t="s">
+        <v>818</v>
+      </c>
+      <c r="C136" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D136" s="36">
+        <v>1350</v>
+      </c>
+      <c r="E136" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A137" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B137" s="35" t="s">
+        <v>817</v>
+      </c>
+      <c r="C137" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D137" s="36">
+        <v>1325</v>
+      </c>
+      <c r="E137" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A138" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B138" s="35" t="s">
+        <v>815</v>
+      </c>
+      <c r="C138" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D138" s="36">
+        <v>1325</v>
+      </c>
+      <c r="E138" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A139" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B139" s="35" t="s">
+        <v>814</v>
+      </c>
+      <c r="C139" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D139" s="36">
+        <v>1300</v>
+      </c>
+      <c r="E139" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A140" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B140" s="35" t="s">
+        <v>812</v>
+      </c>
+      <c r="C140" s="35" t="s">
+        <v>811</v>
+      </c>
+      <c r="D140" s="36">
+        <v>1300</v>
+      </c>
+      <c r="E140" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A141" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B141" s="35" t="s">
+        <v>810</v>
+      </c>
+      <c r="C141" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D141" s="36">
+        <v>1250</v>
+      </c>
+      <c r="E141" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A142" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B142" s="35" t="s">
+        <v>773</v>
+      </c>
+      <c r="C142" s="35" t="s">
+        <v>660</v>
+      </c>
+      <c r="D142" s="36">
+        <v>1170</v>
+      </c>
+      <c r="E142" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A143" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B143" s="35" t="s">
+        <v>760</v>
+      </c>
+      <c r="C143" s="35" t="s">
+        <v>660</v>
+      </c>
+      <c r="D143" s="36">
+        <v>1140</v>
+      </c>
+      <c r="E143" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A144" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B144" s="35" t="s">
+        <v>761</v>
+      </c>
+      <c r="C144" s="35" t="s">
+        <v>660</v>
+      </c>
+      <c r="D144" s="36">
+        <v>1120</v>
+      </c>
+      <c r="E144" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A145" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B145" s="35" t="s">
+        <v>809</v>
+      </c>
+      <c r="C145" s="35" t="s">
+        <v>808</v>
+      </c>
+      <c r="D145" s="36">
+        <v>1050</v>
+      </c>
+      <c r="E145" s="35" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A146" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B146" s="35" t="s">
+        <v>806</v>
+      </c>
+      <c r="C146" s="35" t="s">
+        <v>376</v>
+      </c>
+      <c r="D146" s="36">
+        <v>1040</v>
+      </c>
+      <c r="E146" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A147" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B147" s="35" t="s">
+        <v>805</v>
+      </c>
+      <c r="C147" s="35" t="s">
+        <v>376</v>
+      </c>
+      <c r="D147" s="36">
+        <v>1020</v>
+      </c>
+      <c r="E147" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A148" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B148" s="35" t="s">
+        <v>804</v>
+      </c>
+      <c r="C148" s="35" t="s">
+        <v>376</v>
+      </c>
+      <c r="D148" s="36">
+        <v>1000</v>
+      </c>
+      <c r="E148" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A149" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B149" s="35" t="s">
+        <v>764</v>
+      </c>
+      <c r="C149" s="35" t="s">
+        <v>660</v>
+      </c>
+      <c r="D149" s="36">
+        <v>915</v>
+      </c>
+      <c r="E149" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A150" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B150" s="35" t="s">
+        <v>754</v>
+      </c>
+      <c r="C150" s="35" t="s">
+        <v>660</v>
+      </c>
+      <c r="D150" s="36">
+        <v>910</v>
+      </c>
+      <c r="E150" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A151" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B151" s="35" t="s">
+        <v>803</v>
+      </c>
+      <c r="C151" s="35" t="s">
+        <v>376</v>
+      </c>
+      <c r="D151" s="36">
+        <v>895</v>
+      </c>
+      <c r="E151" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A152" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B152" s="35" t="s">
+        <v>788</v>
+      </c>
+      <c r="C152" s="35" t="s">
+        <v>171</v>
+      </c>
+      <c r="D152" s="36">
+        <v>840</v>
+      </c>
+      <c r="E152" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A153" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B153" s="35" t="s">
+        <v>802</v>
+      </c>
+      <c r="C153" s="35" t="s">
+        <v>376</v>
+      </c>
+      <c r="D153" s="36">
+        <v>835</v>
+      </c>
+      <c r="E153" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A154" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B154" s="35" t="s">
+        <v>769</v>
+      </c>
+      <c r="C154" s="35" t="s">
+        <v>660</v>
+      </c>
+      <c r="D154" s="36">
+        <v>800</v>
+      </c>
+      <c r="E154" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A155" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B155" s="35" t="s">
+        <v>791</v>
+      </c>
+      <c r="C155" s="35" t="s">
+        <v>171</v>
+      </c>
+      <c r="D155" s="36">
+        <v>795</v>
+      </c>
+      <c r="E155" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A156" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B156" s="35" t="s">
+        <v>757</v>
+      </c>
+      <c r="C156" s="35" t="s">
+        <v>660</v>
+      </c>
+      <c r="D156" s="36">
+        <v>790</v>
+      </c>
+      <c r="E156" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A157" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B157" s="35" t="s">
+        <v>776</v>
+      </c>
+      <c r="C157" s="35" t="s">
+        <v>774</v>
+      </c>
+      <c r="D157" s="36">
+        <v>775</v>
+      </c>
+      <c r="E157" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A158" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B158" s="35" t="s">
+        <v>751</v>
+      </c>
+      <c r="C158" s="35" t="s">
+        <v>660</v>
+      </c>
+      <c r="D158" s="36">
+        <v>765</v>
+      </c>
+      <c r="E158" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A159" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B159" s="35" t="s">
+        <v>753</v>
+      </c>
+      <c r="C159" s="35" t="s">
+        <v>660</v>
+      </c>
+      <c r="D159" s="36">
+        <v>755</v>
+      </c>
+      <c r="E159" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A160" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B160" s="35" t="s">
+        <v>772</v>
+      </c>
+      <c r="C160" s="35" t="s">
+        <v>660</v>
+      </c>
+      <c r="D160" s="36">
+        <v>750</v>
+      </c>
+      <c r="E160" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A161" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B161" s="35" t="s">
+        <v>762</v>
+      </c>
+      <c r="C161" s="35" t="s">
+        <v>660</v>
+      </c>
+      <c r="D161" s="36">
+        <v>745</v>
+      </c>
+      <c r="E161" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A162" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B162" s="35" t="s">
+        <v>763</v>
+      </c>
+      <c r="C162" s="35" t="s">
+        <v>660</v>
+      </c>
+      <c r="D162" s="36">
+        <v>740</v>
+      </c>
+      <c r="E162" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A163" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B163" s="35" t="s">
+        <v>777</v>
+      </c>
+      <c r="C163" s="35" t="s">
+        <v>774</v>
+      </c>
+      <c r="D163" s="36">
+        <v>735</v>
+      </c>
+      <c r="E163" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A164" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B164" s="35" t="s">
+        <v>765</v>
+      </c>
+      <c r="C164" s="35" t="s">
+        <v>660</v>
+      </c>
+      <c r="D164" s="36">
+        <v>730</v>
+      </c>
+      <c r="E164" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A165" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B165" s="35" t="s">
+        <v>589</v>
+      </c>
+      <c r="C165" s="35" t="s">
+        <v>376</v>
+      </c>
+      <c r="D165" s="36">
+        <v>730</v>
+      </c>
+      <c r="E165" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A166" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B166" s="35" t="s">
+        <v>797</v>
+      </c>
+      <c r="C166" s="35" t="s">
+        <v>173</v>
+      </c>
+      <c r="D166" s="36">
+        <v>720</v>
+      </c>
+      <c r="E166" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A167" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B167" s="35" t="s">
+        <v>799</v>
+      </c>
+      <c r="C167" s="35" t="s">
+        <v>393</v>
+      </c>
+      <c r="D167" s="36">
+        <v>710</v>
+      </c>
+      <c r="E167" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A168" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B168" s="35" t="s">
+        <v>798</v>
+      </c>
+      <c r="C168" s="35" t="s">
+        <v>376</v>
+      </c>
+      <c r="D168" s="36">
+        <v>705</v>
+      </c>
+      <c r="E168" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A169" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B169" s="35" t="s">
+        <v>781</v>
+      </c>
+      <c r="C169" s="35" t="s">
+        <v>326</v>
+      </c>
+      <c r="D169" s="36">
+        <v>695</v>
+      </c>
+      <c r="E169" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A170" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B170" s="35" t="s">
+        <v>767</v>
+      </c>
+      <c r="C170" s="35" t="s">
+        <v>660</v>
+      </c>
+      <c r="D170" s="36">
+        <v>690</v>
+      </c>
+      <c r="E170" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A171" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B171" s="35" t="s">
+        <v>771</v>
+      </c>
+      <c r="C171" s="35" t="s">
+        <v>660</v>
+      </c>
+      <c r="D171" s="36">
+        <v>685</v>
+      </c>
+      <c r="E171" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A172" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B172" s="35" t="s">
+        <v>795</v>
+      </c>
+      <c r="C172" s="35" t="s">
+        <v>376</v>
+      </c>
+      <c r="D172" s="36">
+        <v>680</v>
+      </c>
+      <c r="E172" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A173" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B173" s="35" t="s">
+        <v>794</v>
+      </c>
+      <c r="C173" s="35" t="s">
+        <v>376</v>
+      </c>
+      <c r="D173" s="36">
+        <v>680</v>
+      </c>
+      <c r="E173" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A174" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B174" s="35" t="s">
+        <v>752</v>
+      </c>
+      <c r="C174" s="35" t="s">
+        <v>660</v>
+      </c>
+      <c r="D174" s="36">
+        <v>675</v>
+      </c>
+      <c r="E174" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A175" s="37">
+        <v>2026</v>
+      </c>
+      <c r="B175" s="35" t="s">
+        <v>793</v>
+      </c>
+      <c r="C175" s="35" t="s">
+        <v>376</v>
+      </c>
+      <c r="D175" s="36">
+        <v>675</v>
+      </c>
+      <c r="E175" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A176">
+        <v>2025</v>
+      </c>
+      <c r="B176" t="s">
+        <v>792</v>
+      </c>
+      <c r="C176" t="s">
+        <v>376</v>
+      </c>
+      <c r="D176" s="34">
+        <v>630</v>
+      </c>
+      <c r="E176" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A177">
+        <v>2024</v>
+      </c>
+      <c r="B177" t="s">
+        <v>784</v>
+      </c>
+      <c r="C177" t="s">
+        <v>171</v>
+      </c>
+      <c r="D177" s="34">
+        <v>595</v>
+      </c>
+      <c r="E177" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A178">
+        <v>2023</v>
+      </c>
+      <c r="B178" t="s">
+        <v>780</v>
+      </c>
+      <c r="C178" t="s">
+        <v>326</v>
+      </c>
+      <c r="D178" s="34">
+        <v>590</v>
+      </c>
+      <c r="E178" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A179">
+        <v>2024</v>
+      </c>
+      <c r="B179" t="s">
+        <v>766</v>
+      </c>
+      <c r="C179" t="s">
+        <v>660</v>
+      </c>
+      <c r="D179" s="34">
+        <v>550</v>
+      </c>
+      <c r="E179" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A180">
+        <v>2025</v>
+      </c>
+      <c r="B180" t="s">
+        <v>759</v>
+      </c>
+      <c r="C180" t="s">
+        <v>660</v>
+      </c>
+      <c r="D180" s="34">
+        <v>655</v>
+      </c>
+      <c r="E180" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A181">
+        <v>2024</v>
+      </c>
+      <c r="B181" t="s">
+        <v>775</v>
+      </c>
+      <c r="C181" t="s">
+        <v>774</v>
+      </c>
+      <c r="D181" s="34">
+        <v>565</v>
+      </c>
+      <c r="E181" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A182">
+        <v>2025</v>
+      </c>
+      <c r="B182" t="s">
+        <v>755</v>
+      </c>
+      <c r="C182" t="s">
+        <v>660</v>
+      </c>
+      <c r="D182" s="34">
+        <v>640</v>
+      </c>
+      <c r="E182" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A183">
+        <v>2025</v>
+      </c>
+      <c r="B183" t="s">
+        <v>770</v>
+      </c>
+      <c r="C183" t="s">
+        <v>660</v>
+      </c>
+      <c r="D183" s="34">
+        <v>645</v>
+      </c>
+      <c r="E183" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A184">
+        <v>2025</v>
+      </c>
+      <c r="B184" t="s">
+        <v>790</v>
+      </c>
+      <c r="C184" t="s">
+        <v>164</v>
+      </c>
+      <c r="D184" s="34">
+        <v>750</v>
+      </c>
+      <c r="E184" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A185">
+        <v>2024</v>
+      </c>
+      <c r="B185" t="s">
+        <v>789</v>
+      </c>
+      <c r="C185" t="s">
+        <v>173</v>
+      </c>
+      <c r="D185" s="34">
+        <v>610</v>
+      </c>
+      <c r="E185" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A186">
+        <v>2024</v>
+      </c>
+      <c r="B186" t="s">
+        <v>768</v>
+      </c>
+      <c r="C186" t="s">
+        <v>660</v>
+      </c>
+      <c r="D186" s="34">
+        <v>560</v>
+      </c>
+      <c r="E186" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A187">
+        <v>2023</v>
+      </c>
+      <c r="B187" t="s">
+        <v>779</v>
+      </c>
+      <c r="C187" t="s">
+        <v>154</v>
+      </c>
+      <c r="D187" s="34">
+        <v>535</v>
+      </c>
+      <c r="E187" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A188">
+        <v>2023</v>
+      </c>
+      <c r="B188" t="s">
+        <v>786</v>
+      </c>
+      <c r="C188" t="s">
+        <v>171</v>
+      </c>
+      <c r="D188" s="34">
+        <v>530</v>
+      </c>
+      <c r="E188" s="35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>